<commit_message>
Tailor faculty requests SR25-style and add scoring/target review formulas
- Faculty request wording rewritten (faculty_requests.py), pointing to each
  faculty's end-2025 response; original wording kept in a Request wording log tab
- Add A1. Data scoring, 0.5 Target Check and T2. Single target review tabs,
  adapted from the SR25 master formulas
- Drop 'Qualitative target?' column from the requirements matrix

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXuBp5SMoG4pD1jWH8rtoe
</commit_message>
<xml_diff>
--- a/output/central_unit_requests/CFOG - end-2026 sustainability reporting request.xlsx
+++ b/output/central_unit_requests/CFOG - end-2026 sustainability reporting request.xlsx
@@ -1508,7 +1508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E9"/>
+  <dimension ref="B1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1532,6 +1532,21 @@
           <t>Y/N</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Target status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Response count</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -1554,6 +1569,17 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
@@ -1576,6 +1602,17 @@
           <t>No</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -1598,6 +1635,17 @@
           <t>TBC</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
@@ -1609,6 +1657,17 @@
         <is>
           <t>Support meeting</t>
         </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Not yet started</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Add each unit's SR25 responses as a linked tab in its request workbook
- New '3. SR25 responses' tab per faculty/central unit request, read from the
  matching SR25 master tab (faculties, CD, CFOG, Business Services, Chancellery
  Research & Enterprise, Legal and Risk); CIOG noted as new
- Column H 'Related SR25 ref' now visible and hyperlinked to the full response;
  request text points to it
- Central units get related SR25 refs and the opening pointer line too

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXuBp5SMoG4pD1jWH8rtoe
</commit_message>
<xml_diff>
--- a/output/central_unit_requests/CFOG - end-2026 sustainability reporting request.xlsx
+++ b/output/central_unit_requests/CFOG - end-2026 sustainability reporting request.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Reporting template" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. OPTIONAL highlighted stories" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. SR25 responses" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +41,32 @@
       <b val="1"/>
       <color rgb="00002060"/>
       <sz val="22"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Aptos"/>
@@ -80,12 +107,6 @@
       <sz val="14"/>
     </font>
     <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
       <name val="Aptos Narrow"/>
       <b val="1"/>
       <color rgb="000E2841"/>
@@ -100,11 +121,9 @@
     <font>
       <name val="Aptos Narrow"/>
       <b val="1"/>
+      <color rgb="000563C1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <sz val="11"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="7">
@@ -116,7 +135,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="000B3040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C1E4F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -126,17 +155,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFC000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C1E4F5"/>
       </patternFill>
     </fill>
   </fills>
@@ -147,12 +166,6 @@
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="medium"/>
-      <right style="medium"/>
-      <top style="medium"/>
-      <bottom style="medium"/>
     </border>
     <border>
       <left style="thin">
@@ -168,62 +181,73 @@
         <color rgb="00808080"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -599,7 +623,7 @@
     <col width="38" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
-    <col hidden="1" outlineLevel="1" width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="9" max="9"/>
     <col hidden="1" outlineLevel="1" width="50" customWidth="1" min="10" max="10"/>
     <col hidden="1" outlineLevel="1" width="24" customWidth="1" min="11" max="11"/>
@@ -650,7 +674,7 @@
 • Provide commentary on progress towards each target (Column M or N)
 • Provide supporting documentation if required (Column O), including links to images
 • Note the source of your information and any limitations (Column P), then confirm the information is accurate (Columns Q–R)
-• Your end-2025 responses (where a related target existed) can be viewed by clicking the [+] icon above Columns H–K
+• Where a related end-2025 target existed, click the ref in Column H to see your full SR25 response (Tab 3)
 • Use Tab 2 of this spreadsheet to highlight key sustainability stories (optional)
 • 2026 is a transition year: Sustainability 2030 launched ~20 October 2026, so report on activity across all of 2026 and any early actions since launch.
 • Due: Friday 15 January 2027 (TBC). Questions: Sustainability Strategy team (sustainability-strategy@unimelb.edu.au – TBC)</t>
@@ -728,7 +752,7 @@
       </c>
       <c r="H13" s="12" t="inlineStr">
         <is>
-          <t>End-2025 reporting (for reference – click [+] above to expand)</t>
+          <t>End-2025 reporting (click the ref to see your full SR25 response; [+] above expands a summary)</t>
         </is>
       </c>
       <c r="L13" s="13" t="inlineStr">
@@ -904,7 +928,11 @@
           <t>We will report on ways the University is making research practices more sustainable in the 2026 Sustainability Report, and share practical examples (e.g. green labs) across faculties.</t>
         </is>
       </c>
-      <c r="H16" s="19" t="inlineStr"/>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>N/A – new indicator</t>
+        </is>
+      </c>
       <c r="I16" s="19" t="inlineStr"/>
       <c r="J16" s="19" t="inlineStr"/>
       <c r="K16" s="19" t="inlineStr"/>
@@ -947,7 +975,11 @@
           <t>We will report on the high-risk procurement categories or suppliers prioritised for nature-impact management, and related actions, in the 2026 Sustainability Report.</t>
         </is>
       </c>
-      <c r="H17" s="19" t="inlineStr"/>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>N/A – new indicator</t>
+        </is>
+      </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="19" t="inlineStr"/>
       <c r="K17" s="19" t="inlineStr"/>
@@ -982,7 +1014,8 @@
       </c>
       <c r="F18" s="19" t="inlineStr">
         <is>
-          <t>Maturity score if framework established; % procurement staff trained</t>
+          <t>In end-2025 reporting your area reported on the related SP2030 target 11c(iii) and rated it 'Met or exceeded' (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
+Maturity score if framework established; % procurement staff trained</t>
         </is>
       </c>
       <c r="G18" s="19" t="inlineStr">
@@ -990,9 +1023,23 @@
           <t>We will use case studies (and any maturity score or training data) to show improvement in responsible procurement processes and systems in the 2026 Sustainability Report.</t>
         </is>
       </c>
-      <c r="H18" s="19" t="inlineStr"/>
-      <c r="I18" s="19" t="inlineStr"/>
-      <c r="J18" s="19" t="inlineStr"/>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>11c(iii)
+→ view SR25 response</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="J18" s="19" t="inlineStr">
+        <is>
+          <t>From Matt (20/1/26): This has not changed from prior years, are you able to use what we submitted last report? (RH note: Yes we can use this).
+From Matt (28/1/26): In 2025 we increased the University’s systemic approach e.g. embedding more outcome focus questions in tenders, enhancing Modern Slavery clauses, implementing a system approach to collecting subcontracted impact spend.</t>
+        </is>
+      </c>
       <c r="K18" s="19" t="inlineStr"/>
       <c r="L18" s="19" t="n"/>
       <c r="M18" s="19" t="n"/>
@@ -1025,7 +1072,8 @@
       </c>
       <c r="F19" s="19" t="inlineStr">
         <is>
-          <t>Annual Modern Slavery Statement, with case studies</t>
+          <t>In end-2025 reporting your area reported on the related SP2030 target 11c(i) and rated it 'Met or exceeded' (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
+Annual Modern Slavery Statement, with case studies</t>
         </is>
       </c>
       <c r="G19" s="19" t="inlineStr">
@@ -1033,9 +1081,25 @@
           <t>We will draw on the annual Modern Slavery Statement and case studies to report on the University's approach to modern slavery and human rights risks (timing to be aligned with the Statement).</t>
         </is>
       </c>
-      <c r="H19" s="19" t="inlineStr"/>
-      <c r="I19" s="19" t="inlineStr"/>
-      <c r="J19" s="19" t="inlineStr"/>
+      <c r="H19" s="20" t="inlineStr">
+        <is>
+          <t>11c(i)
+→ view SR25 response</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="J19" s="19" t="inlineStr">
+        <is>
+          <t>From Matt (20/1/26): Link to Annual Modern Slavery Statement; case study excerpt
+Link: https://modernslaveryregister.gov.au/statements/22714/
+We are currently compiling the 2025 statement which will be published in May (2026). 
+In regard to what new information we are Ok with publishing on MS in regard to 2025 our approach is to collate this and have it approved for external consumption via this process.</t>
+        </is>
+      </c>
       <c r="K19" s="19" t="inlineStr"/>
       <c r="L19" s="19" t="n"/>
       <c r="M19" s="19" t="n"/>
@@ -1076,7 +1140,11 @@
           <t>We will report on internal engagement and partnerships contributing to Sustainability 2030 outcomes, and update our record of sustainability-focused communities of practice and contacts across the University.</t>
         </is>
       </c>
-      <c r="H20" s="19" t="inlineStr"/>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>N/A – new indicator</t>
+        </is>
+      </c>
       <c r="I20" s="19" t="inlineStr"/>
       <c r="J20" s="19" t="inlineStr"/>
       <c r="K20" s="19" t="inlineStr"/>
@@ -1119,7 +1187,11 @@
           <t>We will report on how sustainability is integrated into governance and decision-making across faculties and portfolios, and use responses as a baseline for the governance enabler from 2027.</t>
         </is>
       </c>
-      <c r="H21" s="19" t="inlineStr"/>
+      <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>N/A – new indicator</t>
+        </is>
+      </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="19" t="inlineStr"/>
       <c r="K21" s="19" t="inlineStr"/>
@@ -1146,7 +1218,7 @@
       </c>
       <c r="H26" s="12" t="inlineStr">
         <is>
-          <t>End-2025 reporting (for reference – click [+] above to expand)</t>
+          <t>End-2025 reporting (click the ref to see your full SR25 response; [+] above expands a summary)</t>
         </is>
       </c>
       <c r="L26" s="13" t="inlineStr">
@@ -1314,7 +1386,8 @@
       </c>
       <c r="F29" s="19" t="inlineStr">
         <is>
-          <t>Report on relevant sustainability-related investment portfolio metrics and report on how the University has complied with its related obligations</t>
+          <t>In end-2025 reporting your area reported on the related SP2030 target 12b(i) and rated it 'Met or exceeded' (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
+Report on relevant sustainability-related investment portfolio metrics and report on how the University has complied with its related obligations</t>
         </is>
       </c>
       <c r="G29" s="19" t="inlineStr">
@@ -1322,9 +1395,23 @@
           <t>We will report on sustainability-related investment portfolio metrics and the University's compliance with related obligations (e.g. UNPRI) in the Responsible investments section of the 2026 Sustainability Report.</t>
         </is>
       </c>
-      <c r="H29" s="19" t="inlineStr"/>
-      <c r="I29" s="19" t="inlineStr"/>
-      <c r="J29" s="19" t="inlineStr"/>
+      <c r="H29" s="20" t="inlineStr">
+        <is>
+          <t>12b(i)
+→ view SR25 response</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="J29" s="19" t="inlineStr">
+        <is>
+          <t>Since 2022 the University has published its sustainability-related investment portfolio metrics including carbon intensity. Historically this has only applied to Australian &amp; International equities, but from this year we are able to also include Fixed Income &amp; Credit. Other asset classes will be included as the data relating to them becomes available and is considered reasonable. 
+While data and metrics are continuously being refined, we have met our target of enhanced transparent reporting of the investment portfolio.</t>
+        </is>
+      </c>
       <c r="K29" s="19" t="inlineStr"/>
       <c r="L29" s="19" t="n"/>
       <c r="M29" s="19" t="n"/>
@@ -1364,6 +1451,11 @@
       <formula1>=Lists!$C$2:$C$4</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="H18" location="'3. SR25 responses'!B12"/>
+    <hyperlink ref="H19" location="'3. SR25 responses'!B10"/>
+    <hyperlink ref="H29" location="'3. SR25 responses'!B22"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1414,7 +1506,7 @@
           <t>How to use this spreadsheet</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>Please share up to 3 stories from 2026 which highlight your faculty's/portfolio's sustainability progress and/or impact. These stories can directly relate to Sustainability 2030 targets and indicators, or sustainability more generally. Due: Friday 4 December 2026 (TBC) (early submission helps us develop case studies).</t>
         </is>
@@ -1422,47 +1514,47 @@
     </row>
     <row r="6"/>
     <row r="8">
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D8" s="21" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>Related Sustainability 2030 targets (optional)</t>
         </is>
       </c>
-      <c r="E8" s="21" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>Images and other media</t>
         </is>
       </c>
-      <c r="F8" s="21" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>Links and supporting documentation</t>
         </is>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1">
-      <c r="B9" s="22" t="inlineStr"/>
-      <c r="C9" s="22" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr"/>
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>• Please include a brief description of a project or activity that has made a significant contribution to sustainability at the University (up to 250 words)
 • Summarise the benefits. Benefits may relate to operational outcomes, environmental/social outcomes, and sector benefits.</t>
         </is>
       </c>
-      <c r="D9" s="22" t="inlineStr"/>
-      <c r="E9" s="22" t="inlineStr">
+      <c r="D9" s="23" t="inlineStr"/>
+      <c r="E9" s="23" t="inlineStr">
         <is>
           <t>(link to OneDrive/SharePoint files or published online content preferred)</t>
         </is>
       </c>
-      <c r="F9" s="22" t="inlineStr"/>
+      <c r="F9" s="23" t="inlineStr"/>
     </row>
     <row r="10" ht="120" customHeight="1">
       <c r="A10" t="n">
@@ -1711,4 +1803,663 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>↑</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>End-2025 target status assessment and reporting (for reference)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Your SR25 responses – Chief Finance Officer Group (CFOG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>Your responses to the end-2025 reporting request, against the former Sustainability Plan 2030 (SP2030) targets. For reference only – please do not edit. Use the 'Back to request' links to return to the reporting template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>← Back to request</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>SR25 ref</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>SP2030 target</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>2025 reporting request</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Confirmed end-2025 status</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>OPTION 1: Target-level reporting</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>OPTION 2: Indicator-level reporting</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Supporting information/comments</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>Related SR26 indicator(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="160" customHeight="1">
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>2a</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>The University has curated living labs covering the priority areas of this Plan</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Please describe any activities in Procurement which address sustainability issues via collaboration between academic and professional staff.</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>Not provided</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr"/>
+      <c r="G7" s="19" t="inlineStr"/>
+      <c r="H7" s="19" t="inlineStr"/>
+      <c r="I7" s="19" t="inlineStr"/>
+    </row>
+    <row r="8" ht="160" customHeight="1">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>11a(iii)</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>The University has reduced waste to landfill to 10kg per person</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Case studies on end of life pathways for specialist university waste streams in 2025 (e.g. the lab equipment auction organised by Procurement c. 2023)</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>Not provided (as agreed with Sustainability Strategy team)</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>From Jose:
+At the moment we do not track any reduction of waste in our operation. 
+It might be captured during the contract management process, which is done by the business.
+I might be incorrect, but I think there was a push in Technology to reduce packaging of Laptops and/or other technology devices.
+This would sit under Business Services , most likely under Daniel Buttigieg (after the changes coming due to Byron's departure).
+In our space Tom Atta or Peter Sritharan would be able to confirm or guide internally who to talk to to confirm this initiative. The potential suppliers that are doing this are CompNow and/or Citadel or others in the AV Space.</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr"/>
+      <c r="H8" s="19" t="inlineStr"/>
+      <c r="I8" s="19" t="inlineStr"/>
+    </row>
+    <row r="9" ht="160" customHeight="1">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>11b(iv)</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>The University has reduced the flow and improved the circularity of materials passing through the University</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Case studies demonstrating waste and/or circular economy innovation</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>Not provided (as agreed with Sustainability Strategy team)</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>RH note: Not provided, but not critical for reporting.</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr"/>
+      <c r="H9" s="19" t="inlineStr"/>
+      <c r="I9" s="19" t="inlineStr"/>
+    </row>
+    <row r="10" ht="160" customHeight="1">
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>11c(i)</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>The University has principles for ethical and sustainable consumption and service provision embedded into operations and procurement practices</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Link to Annual Modern Slavery Statement; case study excerpt</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>From Matt (20/1/26): Link to Annual Modern Slavery Statement; case study excerpt
+Link: https://modernslaveryregister.gov.au/statements/22714/
+We are currently compiling the 2025 statement which will be published in May (2026). 
+In regard to what new information we are Ok with publishing on MS in regard to 2025 our approach is to collate this and have it approved for external consumption via this process.</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr"/>
+      <c r="H10" s="19" t="inlineStr"/>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>MS1(a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="160" customHeight="1">
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>11c(ii)</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>The University has principles for ethical and sustainable consumption and service provision embedded into operations and procurement practices</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>List of Fair Trade and other relevant third-party certifications</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>Not provided (as agreed with Sustainability Strategy team)</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>RH note: Not provided, but not critical for reporting</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr"/>
+      <c r="H11" s="19" t="inlineStr"/>
+      <c r="I11" s="19" t="inlineStr"/>
+    </row>
+    <row r="12" ht="160" customHeight="1">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>11c(iii)</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>The University has principles for ethical and sustainable consumption and service provision embedded into operations and procurement practices</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Description of the process for integrating supplier code of conduct into procurement practices, and key outcomes from this process.</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>From Matt (20/1/26): This has not changed from prior years, are you able to use what we submitted last report? (RH note: Yes we can use this).
+From Matt (28/1/26): In 2025 we increased the University’s systemic approach e.g. embedding more outcome focus questions in tenders, enhancing Modern Slavery clauses, implementing a system approach to collecting subcontracted impact spend.</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr"/>
+      <c r="H12" s="19" t="inlineStr"/>
+      <c r="I12" s="19" t="inlineStr">
+        <is>
+          <t>RP1(a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="160" customHeight="1">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>11d</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>The University tracks spend with social and Indigenous suppliers, setting targets from 2024</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Dollars spent with suppliers that are classified as social and/or Indigenous supplies (for example, demonstrated by listings on Supply Nation, Social Traders etc) as a percentage of total spend</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>From Matt (20/1/26): As mentioned, due to integration issues with the ERP rollout we will only get direct spend data information at the end of this month (I don’t have an exact ETA yet).
+For the indirect spend (Indigenous/ Social impact suppliers hired via our primary suppliers) this is collated quarterly and Jase is planning on having the 2025 total figures in the next 3 weeks (the construction industry shuts down over Dec/Jan and so we have slower response times). 
+Of note, the University has recently formed an Indigenous Procurement Working Group at the University and given they represent Murmuk Djerring strategy I believe they will want to review and approve any figures being externally reported that are a Murmuk Djerring deliverable.
+From Matt (28/1/26): What we need to get better at is getting closer to hitting our Indigenous and Social impact spend target (3% by 2030). We have recently created an Indigenous Procurement Working Group made up of key University decision makers to better enable progress in this area.</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="inlineStr"/>
+      <c r="H13" s="19" t="inlineStr"/>
+      <c r="I13" s="19" t="inlineStr">
+        <is>
+          <t>RP2(a), RP2(b)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>SR25 ref</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>SP2030 target</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>2025 reporting request</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>Confirmed end-2025 status</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>OPTION 1: Target-level reporting</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>OPTION 2: Indicator-level reporting</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
+        <is>
+          <t>Supporting information/comments</t>
+        </is>
+      </c>
+      <c r="I16" s="14" t="inlineStr">
+        <is>
+          <t>Related SR26 indicator(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="160" customHeight="1">
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>8a(i)</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>The University reaches and maintains a 'high' climate change preparedness level</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Assessment based on the Climate Change Preparedness Framework</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>Not provided</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr"/>
+      <c r="G17" s="19" t="inlineStr"/>
+      <c r="H17" s="19" t="inlineStr"/>
+      <c r="I17" s="19" t="inlineStr"/>
+    </row>
+    <row r="18" ht="160" customHeight="1">
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>8a(ii)</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>The University reaches and maintains a 'high' climate change preparedness level</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Please provide commentary regarding the Portfolio/team's level of climate change preparedness. Refer to the Climate Change Preparedness Framework for guidance: https://www.unimelb.edu.au/sustainabilityreport/domain-3-walking-the-talk-in-our-operations/climate-resilience#progress-1</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>Not provided</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr"/>
+      <c r="G18" s="19" t="inlineStr"/>
+      <c r="H18" s="19" t="inlineStr"/>
+      <c r="I18" s="19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>Treasury and Investments</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>SR25 ref</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>SP2030 target</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>2025 reporting request</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Confirmed end-2025 status</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>OPTION 1: Target-level reporting</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>OPTION 2: Indicator-level reporting</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>Supporting information/comments</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>Related SR26 indicator(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="160" customHeight="1">
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>12b(i)</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>Enhanced transparent reporting of the University’s investment portfolio</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Report on relevant sustainability-related investment portfolio metrics, including carbon intensity</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>Since 2022 the University has published its sustainability-related investment portfolio metrics including carbon intensity. Historically this has only applied to Australian &amp; International equities, but from this year we are able to also include Fixed Income &amp; Credit. Other asset classes will be included as the data relating to them becomes available and is considered reasonable. 
+While data and metrics are continuously being refined, we have met our target of enhanced transparent reporting of the investment portfolio.</t>
+        </is>
+      </c>
+      <c r="G22" s="19" t="inlineStr"/>
+      <c r="H22" s="19" t="inlineStr"/>
+      <c r="I22" s="19" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="160" customHeight="1">
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>12b(ii)</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>Enhanced transparent reporting of the University’s investment portfolio</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>Reporting on how the University has complied with its related obligations</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
+        <is>
+          <t>We have met the targets we set out to achieve in 2022 by being more transparent in our reporting.</t>
+        </is>
+      </c>
+      <c r="G23" s="19" t="inlineStr"/>
+      <c r="H23" s="19" t="inlineStr"/>
+      <c r="I23" s="19" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="25" t="inlineStr">
+        <is>
+          <t>Enterprise Portfolio and Investments</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>SR25 ref</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>SP2030 target</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>2025 reporting request</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>Confirmed end-2025 status</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>OPTION 1: Target-level reporting</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>OPTION 2: Indicator-level reporting</t>
+        </is>
+      </c>
+      <c r="H26" s="14" t="inlineStr">
+        <is>
+          <t>Supporting information/comments</t>
+        </is>
+      </c>
+      <c r="I26" s="14" t="inlineStr">
+        <is>
+          <t>Related SR26 indicator(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="160" customHeight="1">
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>8a(i)</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr">
+        <is>
+          <t>The University reaches and maintains a 'high' climate change preparedness level</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>Assessment based on the Climate Change Preparedness Framework</t>
+        </is>
+      </c>
+      <c r="E27" s="19" t="inlineStr">
+        <is>
+          <t>Not provided</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr"/>
+      <c r="G27" s="19" t="inlineStr"/>
+      <c r="H27" s="19" t="inlineStr"/>
+      <c r="I27" s="19" t="inlineStr"/>
+    </row>
+    <row r="28" ht="160" customHeight="1">
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>8a(ii)</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>The University reaches and maintains a 'high' climate change preparedness level</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>Please provide commentary regarding the Portfolio/team's level of climate change preparedness. Refer to the Climate Change Preparedness Framework for guidance: https://www.unimelb.edu.au/sustainabilityreport/domain-3-walking-the-talk-in-our-operations/climate-resilience#progress-1</t>
+        </is>
+      </c>
+      <c r="E28" s="19" t="inlineStr">
+        <is>
+          <t>Not provided</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr"/>
+      <c r="G28" s="19" t="inlineStr"/>
+      <c r="H28" s="19" t="inlineStr"/>
+      <c r="I28" s="19" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:I3"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B4" location="'1. Reporting template'!A1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Separate quantitative data: purge quant-only rows, map to Databook draft, add unit quant tabs
- Remove 10 quantitative-only indicators from the requirements matrix (and from
  scoring/review tabs); add 'Quantitative component' pointer for mixed indicators
- New '2. Quant coverage' (indicator-level Databook coverage, owner, action) and
  '2b. Databook register' (318 data points with confirmation columns) tabs
- Central unit requests get a '4. Quantitative data' tab in the SR25 'CFOG - Quant.'
  style for the Databook metrics they own; request rows point to it
- quant.py parses the Databook draft (source file kept out of the repo)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXuBp5SMoG4pD1jWH8rtoe
</commit_message>
<xml_diff>
--- a/output/central_unit_requests/CFOG - end-2026 sustainability reporting request.xlsx
+++ b/output/central_unit_requests/CFOG - end-2026 sustainability reporting request.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Reporting template" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. OPTIONAL highlighted stories" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. SR25 responses" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. SR25 responses" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Quantitative data" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,8 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="20">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.##"/>
+  </numFmts>
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,7 +48,14 @@
     <font>
       <name val="Aptos Narrow"/>
       <b val="1"/>
-      <sz val="16"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="000E2841"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Aptos"/>
@@ -54,13 +64,29 @@
       <sz val="12"/>
     </font>
     <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="000E2841"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <name val="Aptos Narrow"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Aptos Narrow"/>
-      <sz val="11"/>
+      <b val="1"/>
+      <sz val="16"/>
     </font>
     <font>
       <name val="Aptos"/>
@@ -97,26 +123,8 @@
     <font>
       <name val="Aptos Narrow"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <b val="1"/>
-      <color rgb="000E2841"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <b val="1"/>
       <color rgb="000E2841"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-      <color rgb="000E2841"/>
-      <sz val="12"/>
     </font>
     <font>
       <name val="Aptos Narrow"/>
@@ -135,12 +143,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="000B3040"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000B3040"/>
+        <fgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -151,11 +164,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
   </fills>
@@ -191,63 +199,72 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="2"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1387,7 +1404,8 @@
       <c r="F29" s="19" t="inlineStr">
         <is>
           <t>In end-2025 reporting your area reported on the related SP2030 target 12b(i) and rated it 'Met or exceeded' (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
-Report on relevant sustainability-related investment portfolio metrics and report on how the University has complied with its related obligations</t>
+Report on relevant sustainability-related investment portfolio metrics and report on how the University has complied with its related obligations
+Quantitative figures for this indicator are requested separately in Tab 4 (Quantitative data).</t>
         </is>
       </c>
       <c r="G29" s="19" t="inlineStr">
@@ -1600,217 +1618,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>End 2026 target status</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Data owner confirms</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Request status</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Y/N</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Target status</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Score</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Response count</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Please select from dropdown</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Not sent</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Met or exceeded</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Met or exceeded</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Sent</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Partially met</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Partially met</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Partially – see comments</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Chased</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Not met</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Not met</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Support meeting</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Not yet started</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Not yet started</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Received</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Under review</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Not required</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2462,4 +2269,1601 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>↑</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>End-2026 target status assessment and reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Quantitative data – Chief Finance Officer Group (CFOG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>These figures feed the Sustainability Databook (the University's authoritative quantitative source). Previous years are shown for context – please do not alter. Please provide the CY2026 value (provisional figures are fine; we will confirm final figures with you in February), the data source, and any change to definition or boundary. Due: Friday 15 January 2027 (TBC).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Context only (please do not alter)</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>Please fill in these cells</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>CY2023</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>CY2024</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>CY2025</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>Data status</t>
+        </is>
+      </c>
+      <c r="K6" s="15" t="inlineStr">
+        <is>
+          <t>CY2026 value</t>
+        </is>
+      </c>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>Data source (file name, link or system)</t>
+        </is>
+      </c>
+      <c r="M6" s="15" t="inlineStr">
+        <is>
+          <t>Change to definition or boundary?</t>
+        </is>
+      </c>
+      <c r="N6" s="15" t="inlineStr">
+        <is>
+          <t>Notes / limitations</t>
+        </is>
+      </c>
+      <c r="O6" s="15" t="inlineStr">
+        <is>
+          <t>Useful case studies</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>No instructions – context only.</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr"/>
+      <c r="D7" s="26" t="inlineStr"/>
+      <c r="E7" s="26" t="inlineStr"/>
+      <c r="F7" s="26" t="inlineStr"/>
+      <c r="G7" s="26" t="inlineStr"/>
+      <c r="H7" s="26" t="inlineStr"/>
+      <c r="I7" s="26" t="inlineStr"/>
+      <c r="J7" s="26" t="inlineStr"/>
+      <c r="K7" s="26" t="inlineStr">
+        <is>
+          <t>Please enter numerical values</t>
+        </is>
+      </c>
+      <c r="L7" s="26" t="inlineStr">
+        <is>
+          <t>Please provide a file name or link to the data source</t>
+        </is>
+      </c>
+      <c r="M7" s="26" t="inlineStr">
+        <is>
+          <t>Describe any change since last year (or 'No change')</t>
+        </is>
+      </c>
+      <c r="N7" s="26" t="inlineStr">
+        <is>
+          <t>Please add any additional notes here</t>
+        </is>
+      </c>
+      <c r="O7" s="26" t="inlineStr">
+        <is>
+          <t>Please provide information on any useful case studies</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>RP2(a)</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>Percentage of Indigeneous spend of total addressable procurement spend</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Total procurement spending</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n"/>
+      <c r="G8" s="27" t="n"/>
+      <c r="H8" s="27" t="n"/>
+      <c r="I8" s="27" t="n"/>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K8" s="19" t="n"/>
+      <c r="L8" s="19" t="n"/>
+      <c r="M8" s="19" t="n"/>
+      <c r="N8" s="19" t="n"/>
+      <c r="O8" s="19" t="n"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>RP2(a)</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr"/>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Total Indigeneous spending</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n"/>
+      <c r="G9" s="27" t="n"/>
+      <c r="H9" s="27" t="n"/>
+      <c r="I9" s="27" t="n"/>
+      <c r="J9" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K9" s="19" t="n"/>
+      <c r="L9" s="19" t="n"/>
+      <c r="M9" s="19" t="n"/>
+      <c r="N9" s="19" t="n"/>
+      <c r="O9" s="19" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>RP2(a)</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr"/>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Percentage of Indigeneous spend of total addressable procurement spend</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="n"/>
+      <c r="G10" s="27" t="n"/>
+      <c r="H10" s="27" t="n"/>
+      <c r="I10" s="27" t="n"/>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K10" s="19" t="n"/>
+      <c r="L10" s="19" t="n"/>
+      <c r="M10" s="19" t="n"/>
+      <c r="N10" s="19" t="n"/>
+      <c r="O10" s="19" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>RP2(b)</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>Percentage of social spend of total addressable procurement spend</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Total procurement spending</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="n"/>
+      <c r="G11" s="27" t="n"/>
+      <c r="H11" s="27" t="n"/>
+      <c r="I11" s="27" t="n"/>
+      <c r="J11" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K11" s="19" t="n"/>
+      <c r="L11" s="19" t="n"/>
+      <c r="M11" s="19" t="n"/>
+      <c r="N11" s="19" t="n"/>
+      <c r="O11" s="19" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>RP2(b)</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr"/>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Total social spending</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="n"/>
+      <c r="G12" s="27" t="n"/>
+      <c r="H12" s="27" t="n"/>
+      <c r="I12" s="27" t="n"/>
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K12" s="19" t="n"/>
+      <c r="L12" s="19" t="n"/>
+      <c r="M12" s="19" t="n"/>
+      <c r="N12" s="19" t="n"/>
+      <c r="O12" s="19" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>RP2(b)</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr"/>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Percentage of Indigeneous spend of total addressable procurement spend</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n"/>
+      <c r="G13" s="27" t="n"/>
+      <c r="H13" s="27" t="n"/>
+      <c r="I13" s="27" t="n"/>
+      <c r="J13" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K13" s="19" t="n"/>
+      <c r="L13" s="19" t="n"/>
+      <c r="M13" s="19" t="n"/>
+      <c r="N13" s="19" t="n"/>
+      <c r="O13" s="19" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>RI1(a)</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>Annual monitoring and reporting on the investment portfolio's net zero transition progress, including tracking the percentage of AUM managed by investment managers aligned with (or commited to net zero by 2050</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Total Asset Under Management (AUM)</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n"/>
+      <c r="G14" s="27" t="n"/>
+      <c r="H14" s="27" t="n"/>
+      <c r="I14" s="27" t="n"/>
+      <c r="J14" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K14" s="19" t="n"/>
+      <c r="L14" s="19" t="n"/>
+      <c r="M14" s="19" t="n"/>
+      <c r="N14" s="19" t="n"/>
+      <c r="O14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>RI1(a)</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr"/>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>AUM managed by Investment Managers aligned with net zero commitment</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n"/>
+      <c r="G15" s="27" t="n"/>
+      <c r="H15" s="27" t="n"/>
+      <c r="I15" s="27" t="n"/>
+      <c r="J15" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K15" s="19" t="n"/>
+      <c r="L15" s="19" t="n"/>
+      <c r="M15" s="19" t="n"/>
+      <c r="N15" s="19" t="n"/>
+      <c r="O15" s="19" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>RI1(a)</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr"/>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Percentage of AUM managed by Investment Managers aligned with net zero commitment</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n"/>
+      <c r="G16" s="27" t="n"/>
+      <c r="H16" s="27" t="n"/>
+      <c r="I16" s="27" t="n"/>
+      <c r="J16" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K16" s="19" t="n"/>
+      <c r="L16" s="19" t="n"/>
+      <c r="M16" s="19" t="n"/>
+      <c r="N16" s="19" t="n"/>
+      <c r="O16" s="19" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>Continuous improvement of the reporting of the University's sustainability-related investment profile metrics, including investment in climate mitigation and transition solutions, and compliance with related obligations (e.g. UNPRI)</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Total Asset Under Management (AUM)</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n"/>
+      <c r="G17" s="27" t="n"/>
+      <c r="H17" s="27" t="n"/>
+      <c r="I17" s="27" t="n"/>
+      <c r="J17" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K17" s="19" t="n"/>
+      <c r="L17" s="19" t="n"/>
+      <c r="M17" s="19" t="n"/>
+      <c r="N17" s="19" t="n"/>
+      <c r="O17" s="19" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr"/>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>AUM invested in climate/transition solution</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n"/>
+      <c r="G18" s="27" t="n"/>
+      <c r="H18" s="27" t="n"/>
+      <c r="I18" s="27" t="n"/>
+      <c r="J18" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K18" s="19" t="n"/>
+      <c r="L18" s="19" t="n"/>
+      <c r="M18" s="19" t="n"/>
+      <c r="N18" s="19" t="n"/>
+      <c r="O18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr"/>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Percentage of AUM invested in climate/transition solution</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="n"/>
+      <c r="G19" s="27" t="n"/>
+      <c r="H19" s="27" t="n"/>
+      <c r="I19" s="27" t="n"/>
+      <c r="J19" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K19" s="19" t="n"/>
+      <c r="L19" s="19" t="n"/>
+      <c r="M19" s="19" t="n"/>
+      <c r="N19" s="19" t="n"/>
+      <c r="O19" s="19" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr"/>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Estimated UoM absolute financed carbon emissions</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="n"/>
+      <c r="G20" s="27" t="n">
+        <v>121733</v>
+      </c>
+      <c r="H20" s="27" t="n">
+        <v>111919</v>
+      </c>
+      <c r="I20" s="27" t="n">
+        <v>123381</v>
+      </c>
+      <c r="J20" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K20" s="19" t="n"/>
+      <c r="L20" s="19" t="n"/>
+      <c r="M20" s="19" t="n"/>
+      <c r="N20" s="19" t="n"/>
+      <c r="O20" s="19" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr"/>
+      <c r="D21" s="28" t="inlineStr">
+        <is>
+          <t>Australian Equities</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n"/>
+      <c r="G21" s="27" t="n">
+        <v>101663</v>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>82052</v>
+      </c>
+      <c r="I21" s="27" t="n">
+        <v>57483</v>
+      </c>
+      <c r="J21" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K21" s="19" t="n"/>
+      <c r="L21" s="19" t="n"/>
+      <c r="M21" s="19" t="n"/>
+      <c r="N21" s="19" t="n"/>
+      <c r="O21" s="19" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr"/>
+      <c r="D22" s="28" t="inlineStr">
+        <is>
+          <t>International Equities</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="n"/>
+      <c r="G22" s="27" t="n">
+        <v>20070</v>
+      </c>
+      <c r="H22" s="27" t="n">
+        <v>29867</v>
+      </c>
+      <c r="I22" s="27" t="n">
+        <v>27910</v>
+      </c>
+      <c r="J22" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K22" s="19" t="n"/>
+      <c r="L22" s="19" t="n"/>
+      <c r="M22" s="19" t="n"/>
+      <c r="N22" s="19" t="n"/>
+      <c r="O22" s="19" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="inlineStr"/>
+      <c r="D23" s="28" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n"/>
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I23" s="27" t="n">
+        <v>9312</v>
+      </c>
+      <c r="J23" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K23" s="19" t="n"/>
+      <c r="L23" s="19" t="n"/>
+      <c r="M23" s="19" t="n"/>
+      <c r="N23" s="19" t="n"/>
+      <c r="O23" s="19" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr"/>
+      <c r="D24" s="28" t="inlineStr">
+        <is>
+          <t>Fixed Interest</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="n"/>
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H24" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I24" s="27" t="n">
+        <v>28676</v>
+      </c>
+      <c r="J24" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K24" s="19" t="n"/>
+      <c r="L24" s="19" t="n"/>
+      <c r="M24" s="19" t="n"/>
+      <c r="N24" s="19" t="n"/>
+      <c r="O24" s="19" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="inlineStr"/>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>Estimated UoM absolute financed carbon emissions intensity</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e / AUD m invested</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n"/>
+      <c r="G25" s="27" t="n">
+        <v>55</v>
+      </c>
+      <c r="H25" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="J25" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K25" s="19" t="n"/>
+      <c r="L25" s="19" t="n"/>
+      <c r="M25" s="19" t="n"/>
+      <c r="N25" s="19" t="n"/>
+      <c r="O25" s="19" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="inlineStr"/>
+      <c r="D26" s="28" t="inlineStr">
+        <is>
+          <t>Australian Equities</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e / AUD m invested</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="n"/>
+      <c r="G26" s="27" t="n">
+        <v>94</v>
+      </c>
+      <c r="H26" s="27" t="n">
+        <v>72</v>
+      </c>
+      <c r="I26" s="27" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="J26" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K26" s="19" t="n"/>
+      <c r="L26" s="19" t="n"/>
+      <c r="M26" s="19" t="n"/>
+      <c r="N26" s="19" t="n"/>
+      <c r="O26" s="19" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr"/>
+      <c r="D27" s="28" t="inlineStr">
+        <is>
+          <t>International Equities</t>
+        </is>
+      </c>
+      <c r="E27" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e / AUD m invested</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="n"/>
+      <c r="G27" s="27" t="n">
+        <v>18</v>
+      </c>
+      <c r="H27" s="27" t="n">
+        <v>26</v>
+      </c>
+      <c r="I27" s="27" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="J27" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K27" s="19" t="n"/>
+      <c r="L27" s="19" t="n"/>
+      <c r="M27" s="19" t="n"/>
+      <c r="N27" s="19" t="n"/>
+      <c r="O27" s="19" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr"/>
+      <c r="D28" s="28" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="E28" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e / AUD m invested</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="n"/>
+      <c r="G28" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H28" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I28" s="27" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="J28" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K28" s="19" t="n"/>
+      <c r="L28" s="19" t="n"/>
+      <c r="M28" s="19" t="n"/>
+      <c r="N28" s="19" t="n"/>
+      <c r="O28" s="19" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="inlineStr"/>
+      <c r="D29" s="28" t="inlineStr">
+        <is>
+          <t>Fixed Interest</t>
+        </is>
+      </c>
+      <c r="E29" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e / AUD m invested</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="n"/>
+      <c r="G29" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H29" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I29" s="27" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="J29" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K29" s="19" t="n"/>
+      <c r="L29" s="19" t="n"/>
+      <c r="M29" s="19" t="n"/>
+      <c r="N29" s="19" t="n"/>
+      <c r="O29" s="19" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="inlineStr"/>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Benchmark financed carbon emissions</t>
+        </is>
+      </c>
+      <c r="E30" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="n"/>
+      <c r="G30" s="27" t="n">
+        <v>103250</v>
+      </c>
+      <c r="H30" s="27" t="n">
+        <v>118609</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>143399</v>
+      </c>
+      <c r="J30" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K30" s="19" t="n"/>
+      <c r="L30" s="19" t="n"/>
+      <c r="M30" s="19" t="n"/>
+      <c r="N30" s="19" t="n"/>
+      <c r="O30" s="19" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="inlineStr"/>
+      <c r="D31" s="28" t="inlineStr">
+        <is>
+          <t>Australian Equities</t>
+        </is>
+      </c>
+      <c r="E31" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="n"/>
+      <c r="G31" s="27" t="n">
+        <v>62433</v>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>76031</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>49827</v>
+      </c>
+      <c r="J31" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K31" s="19" t="n"/>
+      <c r="L31" s="19" t="n"/>
+      <c r="M31" s="19" t="n"/>
+      <c r="N31" s="19" t="n"/>
+      <c r="O31" s="19" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="inlineStr"/>
+      <c r="D32" s="28" t="inlineStr">
+        <is>
+          <t>International Equities</t>
+        </is>
+      </c>
+      <c r="E32" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e</t>
+        </is>
+      </c>
+      <c r="F32" s="27" t="n"/>
+      <c r="G32" s="27" t="n">
+        <v>40817</v>
+      </c>
+      <c r="H32" s="27" t="n">
+        <v>42578</v>
+      </c>
+      <c r="I32" s="27" t="n">
+        <v>34989</v>
+      </c>
+      <c r="J32" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K32" s="19" t="n"/>
+      <c r="L32" s="19" t="n"/>
+      <c r="M32" s="19" t="n"/>
+      <c r="N32" s="19" t="n"/>
+      <c r="O32" s="19" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="inlineStr"/>
+      <c r="D33" s="28" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="E33" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="n"/>
+      <c r="G33" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H33" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I33" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J33" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K33" s="19" t="n"/>
+      <c r="L33" s="19" t="n"/>
+      <c r="M33" s="19" t="n"/>
+      <c r="N33" s="19" t="n"/>
+      <c r="O33" s="19" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="inlineStr"/>
+      <c r="D34" s="28" t="inlineStr">
+        <is>
+          <t>Fixed Interest</t>
+        </is>
+      </c>
+      <c r="E34" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n"/>
+      <c r="G34" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H34" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I34" s="27" t="n">
+        <v>58583</v>
+      </c>
+      <c r="J34" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K34" s="19" t="n"/>
+      <c r="L34" s="19" t="n"/>
+      <c r="M34" s="19" t="n"/>
+      <c r="N34" s="19" t="n"/>
+      <c r="O34" s="19" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr"/>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>Benchmark financed carbon emissions intensity</t>
+        </is>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e / AUD m invested</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="n"/>
+      <c r="G35" s="27" t="n">
+        <v>47</v>
+      </c>
+      <c r="H35" s="27" t="n">
+        <v>51</v>
+      </c>
+      <c r="I35" s="27" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="J35" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K35" s="19" t="n"/>
+      <c r="L35" s="19" t="n"/>
+      <c r="M35" s="19" t="n"/>
+      <c r="N35" s="19" t="n"/>
+      <c r="O35" s="19" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr"/>
+      <c r="D36" s="28" t="inlineStr">
+        <is>
+          <t>Australian Equities</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e / AUD m invested</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="n"/>
+      <c r="G36" s="27" t="n">
+        <v>58</v>
+      </c>
+      <c r="H36" s="27" t="n">
+        <v>67</v>
+      </c>
+      <c r="I36" s="27" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="J36" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K36" s="19" t="n"/>
+      <c r="L36" s="19" t="n"/>
+      <c r="M36" s="19" t="n"/>
+      <c r="N36" s="19" t="n"/>
+      <c r="O36" s="19" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="inlineStr"/>
+      <c r="D37" s="28" t="inlineStr">
+        <is>
+          <t>International Equities</t>
+        </is>
+      </c>
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e / AUD m invested</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="n"/>
+      <c r="G37" s="27" t="n">
+        <v>36</v>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>37</v>
+      </c>
+      <c r="I37" s="27" t="n">
+        <v>26</v>
+      </c>
+      <c r="J37" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K37" s="19" t="n"/>
+      <c r="L37" s="19" t="n"/>
+      <c r="M37" s="19" t="n"/>
+      <c r="N37" s="19" t="n"/>
+      <c r="O37" s="19" t="n"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C38" s="19" t="inlineStr"/>
+      <c r="D38" s="28" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="E38" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e / AUD m invested</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="n"/>
+      <c r="G38" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H38" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I38" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J38" s="19" t="inlineStr">
+        <is>
+          <t>New – no data yet</t>
+        </is>
+      </c>
+      <c r="K38" s="19" t="n"/>
+      <c r="L38" s="19" t="n"/>
+      <c r="M38" s="19" t="n"/>
+      <c r="N38" s="19" t="n"/>
+      <c r="O38" s="19" t="n"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>RI1(b)</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="inlineStr"/>
+      <c r="D39" s="28" t="inlineStr">
+        <is>
+          <t>Fixed Interest</t>
+        </is>
+      </c>
+      <c r="E39" s="19" t="inlineStr">
+        <is>
+          <t>tCO2-e / AUD m invested</t>
+        </is>
+      </c>
+      <c r="F39" s="27" t="n"/>
+      <c r="G39" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H39" s="27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I39" s="27" t="n">
+        <v>112.9</v>
+      </c>
+      <c r="J39" s="19" t="inlineStr">
+        <is>
+          <t>Data held</t>
+        </is>
+      </c>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="n"/>
+      <c r="M39" s="19" t="n"/>
+      <c r="N39" s="19" t="n"/>
+      <c r="O39" s="19" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B3:O3"/>
+    <mergeCell ref="B5:J5"/>
+    <mergeCell ref="K5:O5"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="M8:M40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Please select from the dropdown" type="list">
+      <formula1>"No change,Yes – see notes"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>End 2026 target status</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Data owner confirms</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Request status</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Y/N</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Target status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Response count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Please select from dropdown</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Met or exceeded</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Partially met</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Partially – see comments</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Chased</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Support meeting</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Not yet started</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Not yet started</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Under review</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Not required</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>